<commit_message>
Update in line with latest 1.08 version
</commit_message>
<xml_diff>
--- a/dependencies/genotype_key.xlsx
+++ b/dependencies/genotype_key.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\project\diagnostic_virology_laboratory\MKillian\Analysis\results\influenza\HPAI\hpai_genotyping_blast\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85205CC9-BEE0-44B4-942F-0857CEFFA431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB0E96E-4311-4295-A5A0-775FFD2280DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-255" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$148</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1503" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="248">
   <si>
     <t>Genotype</t>
   </si>
@@ -548,9 +548,6 @@
     <t>Minor98</t>
   </si>
   <si>
-    <t>Minor99</t>
-  </si>
-  <si>
     <t>Minor101</t>
   </si>
   <si>
@@ -620,9 +617,6 @@
     <t>Minor113</t>
   </si>
   <si>
-    <t>Minor114</t>
-  </si>
-  <si>
     <t>Minor118</t>
   </si>
   <si>
@@ -680,9 +674,6 @@
     <t>am12N5</t>
   </si>
   <si>
-    <t>Minor135</t>
-  </si>
-  <si>
     <t>Minor137</t>
   </si>
   <si>
@@ -759,6 +750,36 @@
   </si>
   <si>
     <t>Minor155</t>
+  </si>
+  <si>
+    <t>D1.13</t>
+  </si>
+  <si>
+    <t>D1.14</t>
+  </si>
+  <si>
+    <t>Minor156</t>
+  </si>
+  <si>
+    <t>Minor157</t>
+  </si>
+  <si>
+    <t>Minor158</t>
+  </si>
+  <si>
+    <t>Minor159</t>
+  </si>
+  <si>
+    <t>Minor160</t>
+  </si>
+  <si>
+    <t>Minor161</t>
+  </si>
+  <si>
+    <t>Minor162</t>
+  </si>
+  <si>
+    <t>D1.15</t>
   </si>
 </sst>
 </file>
@@ -1173,7 +1194,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I167"/>
+  <dimension ref="A1:I174"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1675,13 +1696,13 @@
     </row>
     <row r="18" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>10</v>
@@ -1690,10 +1711,10 @@
         <v>10</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>10</v>
@@ -2168,7 +2189,7 @@
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>41</v>
@@ -2197,7 +2218,7 @@
     </row>
     <row r="36" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>160</v>
@@ -2215,7 +2236,7 @@
         <v>36</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>14</v>
@@ -2226,7 +2247,7 @@
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>45</v>
@@ -2244,7 +2265,7 @@
         <v>36</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>14</v>
@@ -2255,7 +2276,7 @@
     </row>
     <row r="38" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>160</v>
@@ -2284,7 +2305,7 @@
     </row>
     <row r="39" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>160</v>
@@ -2313,7 +2334,7 @@
     </row>
     <row r="40" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>45</v>
@@ -2342,7 +2363,7 @@
     </row>
     <row r="41" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>45</v>
@@ -2371,7 +2392,7 @@
     </row>
     <row r="42" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>128</v>
@@ -2389,7 +2410,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>14</v>
@@ -2400,7 +2421,7 @@
     </row>
     <row r="43" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>128</v>
@@ -2427,12 +2448,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>163</v>
+        <v>238</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>14</v>
@@ -2444,10 +2465,10 @@
         <v>14</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>14</v>
@@ -2456,99 +2477,99 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="H45" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I45" s="9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="H46" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I46" s="9" t="s">
-        <v>10</v>
+        <v>247</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="H47" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I47" s="9" t="s">
-        <v>10</v>
+        <v>163</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>10</v>
@@ -2560,7 +2581,7 @@
         <v>10</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>10</v>
@@ -2574,10 +2595,10 @@
     </row>
     <row r="49" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>10</v>
@@ -2589,7 +2610,7 @@
         <v>10</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>10</v>
@@ -2603,10 +2624,10 @@
     </row>
     <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>10</v>
@@ -2618,7 +2639,7 @@
         <v>10</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>10</v>
@@ -2632,7 +2653,7 @@
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>10</v>
@@ -2647,7 +2668,7 @@
         <v>10</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>10</v>
@@ -2661,10 +2682,10 @@
     </row>
     <row r="52" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>10</v>
@@ -2676,7 +2697,7 @@
         <v>10</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>10</v>
@@ -2690,22 +2711,22 @@
     </row>
     <row r="53" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>10</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>10</v>
@@ -2714,18 +2735,18 @@
         <v>10</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D54" s="9" t="s">
         <v>10</v>
@@ -2734,7 +2755,7 @@
         <v>10</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>10</v>
@@ -2748,13 +2769,13 @@
     </row>
     <row r="55" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>10</v>
@@ -2763,10 +2784,10 @@
         <v>10</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="H55" s="9" t="s">
         <v>10</v>
@@ -2777,22 +2798,22 @@
     </row>
     <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E56" s="9" t="s">
         <v>10</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>10</v>
@@ -2801,18 +2822,18 @@
         <v>10</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>10</v>
@@ -2830,18 +2851,18 @@
         <v>10</v>
       </c>
       <c r="I57" s="9" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D58" s="9" t="s">
         <v>10</v>
@@ -2850,10 +2871,10 @@
         <v>10</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>10</v>
@@ -2864,100 +2885,100 @@
     </row>
     <row r="59" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H59" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I59" s="4" t="s">
-        <v>23</v>
+        <v>67</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I59" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H60" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I60" s="4" t="s">
-        <v>24</v>
+        <v>69</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B61" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B61" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D61" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E61" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H61" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I61" s="4" t="s">
+      <c r="D61" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I61" s="9" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>10</v>
@@ -2966,7 +2987,7 @@
         <v>10</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>10</v>
@@ -2980,13 +3001,13 @@
     </row>
     <row r="63" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>24</v>
+        <v>121</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>10</v>
@@ -2995,7 +3016,7 @@
         <v>10</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G63" s="4" t="s">
         <v>10</v>
@@ -3009,7 +3030,7 @@
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>24</v>
@@ -3024,7 +3045,7 @@
         <v>10</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>10</v>
@@ -3033,18 +3054,18 @@
         <v>10</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>10</v>
@@ -3053,7 +3074,7 @@
         <v>10</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="G65" s="4" t="s">
         <v>10</v>
@@ -3067,10 +3088,10 @@
     </row>
     <row r="66" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>24</v>
@@ -3082,7 +3103,7 @@
         <v>10</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>10</v>
@@ -3091,18 +3112,18 @@
         <v>10</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>10</v>
@@ -3111,7 +3132,7 @@
         <v>10</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="G67" s="4" t="s">
         <v>10</v>
@@ -3125,10 +3146,10 @@
     </row>
     <row r="68" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>24</v>
@@ -3140,7 +3161,7 @@
         <v>10</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G68" s="4" t="s">
         <v>10</v>
@@ -3154,10 +3175,10 @@
     </row>
     <row r="69" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>24</v>
@@ -3169,7 +3190,7 @@
         <v>10</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G69" s="4" t="s">
         <v>10</v>
@@ -3178,18 +3199,18 @@
         <v>10</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>10</v>
@@ -3198,7 +3219,7 @@
         <v>10</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>10</v>
@@ -3212,42 +3233,42 @@
     </row>
     <row r="71" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>222</v>
+        <v>10</v>
       </c>
       <c r="H71" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>64</v>
+        <v>24</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>10</v>
@@ -3256,7 +3277,7 @@
         <v>10</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>10</v>
@@ -3270,13 +3291,13 @@
     </row>
     <row r="73" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>88</v>
+        <v>32</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>10</v>
@@ -3285,7 +3306,7 @@
         <v>10</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G73" s="4" t="s">
         <v>10</v>
@@ -3299,42 +3320,42 @@
     </row>
     <row r="74" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="C74" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D74" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D74" s="4" t="s">
-        <v>10</v>
-      </c>
       <c r="E74" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>10</v>
+        <v>219</v>
       </c>
       <c r="H74" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>10</v>
@@ -3343,7 +3364,7 @@
         <v>10</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>10</v>
@@ -3352,18 +3373,18 @@
         <v>10</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>94</v>
+        <v>64</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>10</v>
@@ -3372,7 +3393,7 @@
         <v>10</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>10</v>
@@ -3386,13 +3407,13 @@
     </row>
     <row r="77" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="D77" s="4" t="s">
         <v>10</v>
@@ -3415,13 +3436,13 @@
     </row>
     <row r="78" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>10</v>
@@ -3439,102 +3460,102 @@
         <v>10</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G79" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I79" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G81" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B79" s="4" t="s">
+      <c r="B82" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F79" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G79" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H79" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I79" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E80" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F80" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G80" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H80" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I80" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E81" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F81" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G81" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H81" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I81" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B82" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>24</v>
@@ -3546,7 +3567,7 @@
         <v>10</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="G82" s="4" t="s">
         <v>10</v>
@@ -3560,42 +3581,42 @@
     </row>
     <row r="83" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B83" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C83" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D83" s="4" t="s">
+      <c r="G83" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I83" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="E83" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F83" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G83" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H83" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I83" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="84" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>10</v>
@@ -3604,7 +3625,7 @@
         <v>10</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>91</v>
+        <v>33</v>
       </c>
       <c r="G84" s="4" t="s">
         <v>10</v>
@@ -3618,22 +3639,22 @@
     </row>
     <row r="85" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>112</v>
+        <v>10</v>
       </c>
       <c r="E85" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>10</v>
@@ -3647,22 +3668,22 @@
     </row>
     <row r="86" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G86" s="4" t="s">
         <v>10</v>
@@ -3671,18 +3692,18 @@
         <v>10</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
     </row>
     <row r="87" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>10</v>
@@ -3691,7 +3712,7 @@
         <v>10</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>10</v>
@@ -3705,71 +3726,71 @@
     </row>
     <row r="88" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B88" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D88" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C88" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>10</v>
-      </c>
       <c r="E88" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>113</v>
+        <v>10</v>
       </c>
       <c r="H88" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="89" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>115</v>
+        <v>45</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>116</v>
+        <v>39</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H89" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="90" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D90" s="4" t="s">
         <v>10</v>
@@ -3778,7 +3799,7 @@
         <v>10</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>10</v>
@@ -3792,68 +3813,68 @@
     </row>
     <row r="91" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="C91" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I91" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="D91" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E91" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F91" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G91" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H91" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I91" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="92" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>23</v>
+        <v>115</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H92" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>115</v>
+        <v>43</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>39</v>
@@ -3865,7 +3886,7 @@
         <v>10</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>10</v>
@@ -3879,10 +3900,10 @@
     </row>
     <row r="94" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>128</v>
+        <v>32</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>39</v>
@@ -3908,187 +3929,187 @@
     </row>
     <row r="95" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>120</v>
+        <v>23</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>12</v>
+        <v>124</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="96" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>36</v>
+        <v>115</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E96" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>94</v>
+        <v>33</v>
       </c>
       <c r="G96" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H96" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>112</v>
+        <v>39</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H97" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>43</v>
+        <v>120</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H98" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H99" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>39</v>
+        <v>115</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>112</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H100" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I100" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>120</v>
+        <v>43</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>10</v>
@@ -4097,7 +4118,7 @@
         <v>10</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>10</v>
@@ -4111,13 +4132,13 @@
     </row>
     <row r="102" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B102" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C102" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>10</v>
@@ -4126,7 +4147,7 @@
         <v>10</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>10</v>
@@ -4140,100 +4161,100 @@
     </row>
     <row r="103" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E103" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F103" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G103" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I103" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F104" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G104" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H104" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G105" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I105" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B106" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C103" s="4" t="s">
+      <c r="C106" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E103" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F103" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G103" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H103" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I103" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C104" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D104" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E104" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F104" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G104" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H104" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I104" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B105" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C105" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D105" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E105" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F105" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G105" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H105" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I105" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A106" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C106" s="4" t="s">
-        <v>116</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>10</v>
@@ -4242,7 +4263,7 @@
         <v>12</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="G106" s="4" t="s">
         <v>12</v>
@@ -4254,55 +4275,55 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>145</v>
+        <v>45</v>
       </c>
       <c r="C107" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F107" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G107" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I107" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C108" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D107" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E107" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F107" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G107" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H107" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I107" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A108" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B108" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C108" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="D108" s="4" t="s">
+      <c r="D108" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E108" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F108" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="G108" s="4" t="s">
+      <c r="F108" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G108" s="6" t="s">
         <v>10</v>
       </c>
       <c r="H108" s="4" t="s">
@@ -4314,128 +4335,128 @@
     </row>
     <row r="109" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B109" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>39</v>
+        <v>116</v>
       </c>
       <c r="D109" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="G109" s="4" t="s">
-        <v>148</v>
+        <v>12</v>
       </c>
       <c r="H109" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I109" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C110" s="9" t="s">
-        <v>121</v>
+        <v>145</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G110" s="6" t="s">
-        <v>12</v>
+        <v>33</v>
+      </c>
+      <c r="G110" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="H110" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I110" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="111" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>120</v>
+        <v>43</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G111" s="6" t="s">
-        <v>12</v>
+        <v>124</v>
+      </c>
+      <c r="G111" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="H111" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I111" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="112" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B112" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C112" s="9" t="s">
-        <v>156</v>
+      <c r="C112" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>12</v>
+        <v>148</v>
       </c>
       <c r="H112" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I112" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="113" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B113" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C113" s="4" t="s">
+      <c r="C113" s="9" t="s">
         <v>121</v>
       </c>
       <c r="D113" s="4" t="s">
@@ -4445,7 +4466,7 @@
         <v>12</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G113" s="6" t="s">
         <v>12</v>
@@ -4459,13 +4480,13 @@
     </row>
     <row r="114" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C114" s="4" t="s">
-        <v>12</v>
+        <v>152</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>121</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>10</v>
@@ -4474,36 +4495,36 @@
         <v>12</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="G114" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G114" s="6" t="s">
         <v>12</v>
       </c>
       <c r="H114" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I114" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="115" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B115" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C115" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C115" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="D115" s="4" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="E115" s="4" t="s">
         <v>12</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="G115" s="4" t="s">
         <v>12</v>
@@ -4517,24 +4538,24 @@
     </row>
     <row r="116" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B116" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>112</v>
+        <v>65</v>
       </c>
       <c r="E116" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F116" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="G116" s="4" t="s">
+      <c r="F116" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G116" s="6" t="s">
         <v>12</v>
       </c>
       <c r="H116" s="4" t="s">
@@ -4546,115 +4567,115 @@
     </row>
     <row r="117" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="B117" s="4" t="s">
-        <v>45</v>
+        <v>155</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>156</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>145</v>
+        <v>12</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="G117" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H117" s="4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="I117" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="118" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>23</v>
+        <v>156</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="G118" s="4" t="s">
-        <v>161</v>
+        <v>12</v>
       </c>
       <c r="H118" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I118" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="119" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>39</v>
+        <v>112</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F119" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G119" s="3" t="s">
-        <v>161</v>
+        <v>12</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G119" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="H119" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I119" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="120" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="E120" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>116</v>
+        <v>14</v>
       </c>
       <c r="G120" s="4" t="s">
-        <v>172</v>
+        <v>14</v>
       </c>
       <c r="H120" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I120" s="4" t="s">
         <v>14</v>
@@ -4662,10 +4683,10 @@
     </row>
     <row r="121" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
-        <v>170</v>
+        <v>184</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>14</v>
@@ -4679,7 +4700,7 @@
       <c r="F121" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G121" s="3" t="s">
+      <c r="G121" s="4" t="s">
         <v>161</v>
       </c>
       <c r="H121" s="4" t="s">
@@ -4689,9 +4710,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="4" t="s">
         <v>160</v>
@@ -4706,10 +4727,10 @@
         <v>14</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G122" s="4" t="s">
-        <v>173</v>
+        <v>14</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>161</v>
       </c>
       <c r="H122" s="4" t="s">
         <v>14</v>
@@ -4718,27 +4739,27 @@
         <v>14</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C123" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E123" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="G123" s="4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="H123" s="4" t="s">
         <v>14</v>
@@ -4749,25 +4770,25 @@
     </row>
     <row r="124" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="C124" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E124" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="H124" s="4" t="s">
         <v>14</v>
@@ -4778,16 +4799,16 @@
     </row>
     <row r="125" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C125" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="E125" s="4" t="s">
         <v>14</v>
@@ -4796,7 +4817,7 @@
         <v>36</v>
       </c>
       <c r="G125" s="4" t="s">
-        <v>14</v>
+        <v>178</v>
       </c>
       <c r="H125" s="4" t="s">
         <v>14</v>
@@ -4807,10 +4828,10 @@
     </row>
     <row r="126" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="C126" s="4" t="s">
         <v>14</v>
@@ -4822,7 +4843,7 @@
         <v>14</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="G126" s="4" t="s">
         <v>14</v>
@@ -4836,103 +4857,103 @@
     </row>
     <row r="127" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B127" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C127" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D127" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D127" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E127" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F127" s="3" t="s">
+      <c r="E127" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F127" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G127" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="H127" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I127" s="3" t="s">
+      <c r="G127" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H127" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I127" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="128" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B128" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D128" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E128" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F128" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G128" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H128" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I128" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H128" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I128" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="129" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B129" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="H129" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I129" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B130" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C129" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D129" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E129" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F129" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="G129" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H129" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I129" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="130" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A130" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="C130" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E130" s="3" t="s">
         <v>14</v>
@@ -4941,85 +4962,85 @@
         <v>36</v>
       </c>
       <c r="G130" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I130" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G131" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="H130" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I130" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="131" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A131" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="B131" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="C131" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D131" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E131" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F131" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G131" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="H131" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I131" s="4" t="s">
+      <c r="H131" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I131" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="132" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B132" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C132" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D132" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E132" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F132" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F132" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G132" s="4" t="s">
+      <c r="G132" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="H132" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I132" s="4" t="s">
+      <c r="H132" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I132" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="133" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B133" s="4" t="s">
         <v>160</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>14</v>
+        <v>94</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>14</v>
@@ -5039,16 +5060,16 @@
     </row>
     <row r="134" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="C134" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>14</v>
@@ -5068,16 +5089,16 @@
     </row>
     <row r="135" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="E135" s="4" t="s">
         <v>14</v>
@@ -5097,16 +5118,16 @@
     </row>
     <row r="136" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B136" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>160</v>
+        <v>14</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="E136" s="4" t="s">
         <v>14</v>
@@ -5126,22 +5147,22 @@
     </row>
     <row r="137" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B137" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C137" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C137" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="D137" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E137" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>88</v>
+        <v>36</v>
       </c>
       <c r="G137" s="4" t="s">
         <v>161</v>
@@ -5155,13 +5176,13 @@
     </row>
     <row r="138" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>164</v>
+        <v>14</v>
       </c>
       <c r="D138" s="4" t="s">
         <v>39</v>
@@ -5170,7 +5191,7 @@
         <v>14</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="G138" s="4" t="s">
         <v>161</v>
@@ -5179,18 +5200,18 @@
         <v>14</v>
       </c>
       <c r="I138" s="4" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="139" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>160</v>
+        <v>45</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D139" s="4" t="s">
         <v>39</v>
@@ -5199,7 +5220,7 @@
         <v>14</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="G139" s="4" t="s">
         <v>161</v>
@@ -5208,18 +5229,18 @@
         <v>14</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="140" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B140" s="4" t="s">
         <v>160</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>14</v>
+        <v>167</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>39</v>
@@ -5228,7 +5249,7 @@
         <v>14</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="G140" s="4" t="s">
         <v>161</v>
@@ -5242,7 +5263,7 @@
     </row>
     <row r="141" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B141" s="4" t="s">
         <v>160</v>
@@ -5257,7 +5278,7 @@
         <v>14</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>161</v>
@@ -5271,22 +5292,22 @@
     </row>
     <row r="142" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="C142" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="E142" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="G142" s="4" t="s">
         <v>161</v>
@@ -5300,22 +5321,22 @@
     </row>
     <row r="143" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>120</v>
+        <v>45</v>
       </c>
       <c r="C143" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="E143" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>161</v>
@@ -5329,22 +5350,22 @@
     </row>
     <row r="144" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C144" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="E144" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="G144" s="4" t="s">
         <v>161</v>
@@ -5358,22 +5379,22 @@
     </row>
     <row r="145" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="C145" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D145" s="3" t="s">
-        <v>99</v>
+      <c r="D145" s="4" t="s">
+        <v>91</v>
       </c>
       <c r="E145" s="4" t="s">
         <v>14</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>36</v>
+        <v>94</v>
       </c>
       <c r="G145" s="4" t="s">
         <v>161</v>
@@ -5387,7 +5408,7 @@
     </row>
     <row r="146" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B146" s="4" t="s">
         <v>160</v>
@@ -5395,8 +5416,8 @@
       <c r="C146" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D146" s="4" t="s">
-        <v>88</v>
+      <c r="D146" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="E146" s="4" t="s">
         <v>14</v>
@@ -5416,7 +5437,7 @@
     </row>
     <row r="147" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B147" s="4" t="s">
         <v>160</v>
@@ -5425,7 +5446,7 @@
         <v>14</v>
       </c>
       <c r="D147" s="4" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="E147" s="4" t="s">
         <v>14</v>
@@ -5445,16 +5466,16 @@
     </row>
     <row r="148" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>39</v>
+        <v>116</v>
       </c>
       <c r="E148" s="4" t="s">
         <v>14</v>
@@ -5474,7 +5495,7 @@
     </row>
     <row r="149" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B149" s="4" t="s">
         <v>160</v>
@@ -5503,7 +5524,7 @@
     </row>
     <row r="150" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B150" s="4" t="s">
         <v>45</v>
@@ -5532,7 +5553,7 @@
     </row>
     <row r="151" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B151" s="4" t="s">
         <v>160</v>
@@ -5561,7 +5582,7 @@
     </row>
     <row r="152" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B152" s="4" t="s">
         <v>45</v>
@@ -5579,7 +5600,7 @@
         <v>128</v>
       </c>
       <c r="G152" s="4" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="H152" s="4" t="s">
         <v>14</v>
@@ -5590,7 +5611,7 @@
     </row>
     <row r="153" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B153" s="4" t="s">
         <v>32</v>
@@ -5619,7 +5640,7 @@
     </row>
     <row r="154" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B154" s="4" t="s">
         <v>160</v>
@@ -5648,7 +5669,7 @@
     </row>
     <row r="155" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B155" s="4" t="s">
         <v>160</v>
@@ -5666,7 +5687,7 @@
         <v>36</v>
       </c>
       <c r="G155" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H155" s="4" t="s">
         <v>14</v>
@@ -5677,7 +5698,7 @@
     </row>
     <row r="156" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B156" s="4" t="s">
         <v>128</v>
@@ -5695,7 +5716,7 @@
         <v>112</v>
       </c>
       <c r="G156" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H156" s="4" t="s">
         <v>14</v>
@@ -5706,7 +5727,7 @@
     </row>
     <row r="157" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B157" s="4" t="s">
         <v>128</v>
@@ -5735,7 +5756,7 @@
     </row>
     <row r="158" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B158" s="4" t="s">
         <v>160</v>
@@ -5764,7 +5785,7 @@
     </row>
     <row r="159" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B159" s="4" t="s">
         <v>160</v>
@@ -5793,7 +5814,7 @@
     </row>
     <row r="160" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B160" s="4" t="s">
         <v>45</v>
@@ -5822,7 +5843,7 @@
     </row>
     <row r="161" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B161" s="4" t="s">
         <v>160</v>
@@ -5851,7 +5872,7 @@
     </row>
     <row r="162" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B162" s="4" t="s">
         <v>160</v>
@@ -5869,7 +5890,7 @@
         <v>83</v>
       </c>
       <c r="G162" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H162" s="4" t="s">
         <v>14</v>
@@ -5880,7 +5901,7 @@
     </row>
     <row r="163" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B163" s="4" t="s">
         <v>160</v>
@@ -5898,7 +5919,7 @@
         <v>23</v>
       </c>
       <c r="G163" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="H163" s="4" t="s">
         <v>14</v>
@@ -5909,7 +5930,7 @@
     </row>
     <row r="164" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B164" s="4" t="s">
         <v>45</v>
@@ -5938,7 +5959,7 @@
     </row>
     <row r="165" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B165" s="4" t="s">
         <v>160</v>
@@ -5967,7 +5988,7 @@
     </row>
     <row r="166" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B166" s="4" t="s">
         <v>45</v>
@@ -5996,7 +6017,7 @@
     </row>
     <row r="167" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B167" s="4" t="s">
         <v>160</v>
@@ -6023,9 +6044,212 @@
         <v>14</v>
       </c>
     </row>
+    <row r="168" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A168" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D168" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E168" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G168" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H168" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I168" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C169" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D169" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E169" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F169" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G169" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H169" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I169" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C170" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D170" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E170" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F170" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G170" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H170" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I170" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C171" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D171" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E171" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F171" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G171" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H171" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I171" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A172" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C172" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D172" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E172" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F172" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G172" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H172" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I172" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A173" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C173" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D173" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E173" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F173" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G173" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H173" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I173" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A174" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C174" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D174" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E174" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F174" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G174" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H174" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I174" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I121">
-    <sortCondition ref="A2:A121"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I123">
+    <sortCondition ref="A2:A123"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>